<commit_message>
repo: no license file; local tooling and machine paths out of the published tree
- LICENSE and apps/easi/LICENSE are removed, and the EASI README drops its
  License section. Third-party notices (vendored libraries, the DejaVu font)
  stay as their licenses require.
- Local editor and tooling files are no longer tracked, and the ignore files
  stop naming them.
- The library provenance records drop two unused run-operator fields, and
  provenance.py no longer writes them. The inputs digest never read them, so
  every recorded digest still reproduces.
- Script docstrings and READMEs point at the repo's own .venv and data
  instead of retired local folders, and no longer cite internal notes.
- STAF_Logo.png and the Wisconsin SQT template lose embedded editor
  metadata. The image's pixels and the workbook's cells are unchanged; the
  SQT registry records the template's new checksum.
</commit_message>
<xml_diff>
--- a/apps/stream-curves/data/templates/WISQT_Reference_Curves.xlsx
+++ b/apps/stream-curves/data/templates/WISQT_Reference_Curves.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\Work\stream-curves-claude\docs\Completed_SQTs\Stream_Quantification_Tool_Ref_Curves\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB60031A-110A-4AC5-A9CB-E5487FB34A1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2070" windowWidth="38640" windowHeight="21120" tabRatio="479" xr2:uid="{AA844D8B-4DC0-4502-BDB2-641660958C8F}"/>

</xml_diff>